<commit_message>
Release v1.1: Improved analysis accuracy for Ürün Miktarı and Saklama Koşulu, added PDF zoom controls, and UI refinements.
</commit_message>
<xml_diff>
--- a/Kural.xlsx
+++ b/Kural.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vande\Desktop\Humanis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8AEE61B-4C72-44AF-8772-3B4FFE0860BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AE338D6-A1AE-4315-96B1-F2D877556C2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="465" yWindow="120" windowWidth="21960" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -224,10 +224,10 @@
     <t xml:space="preserve">25°C-25°C’nin altındaki oda sıcaklığında saklanmalıdır-25°C altında saklayınız-25°C altındaki oda sıcaklığında, kuru bir yerde saklayınız-25 °C’nin altındaki oda sıcaklığında saklayınız.-30°C altındaki oda sıcaklığında saklayınız. Orijinal ambalajında saklayınız. </t>
   </si>
   <si>
-    <t>en çok  25°C  veya 30°C kelimeleriyle kullanılır.%99 25°C kelimesiyle birlikte yazılır.Saklamaya yönelik özel uyarılar: ","saklanması ","’ın saklanması" başlığı altında olur.Çoğunlukla son sayfalarda oluyor.</t>
-  </si>
-  <si>
     <t xml:space="preserve">20 tablet-ASPİRİN, 20 tabletlik ambalajlarda sunulur. -20 veya 30 tablet içeren blister ambalajlarda.-4 adet kapsül ve 8 adet kapsül olmak üzere iki ayrı ambalaj formu mevcuttur. -A-FERİN kapsül 20-30 kapsül içeren blister ambalajlarda kullanıma sunulmuştur. -10 veya 20 tabletlik ambalaj miktarlarında bulunmaktadır. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">en çok  25°C  veya 30°C kelimeleriyle kullanılır.%99 25°C kelimesiyle birlikte yazılır.Saklamaya yönelik özel uyarılar: ","saklanması ","’ın saklanması" başlığı altında olur.Çoğunlukla son sayfalarda oluyor. ONCEAİR'in saklanması gibi başlık altında olur. </t>
   </si>
 </sst>
 </file>
@@ -627,7 +627,7 @@
         <v>59</v>
       </c>
       <c r="C5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -635,7 +635,7 @@
         <v>60</v>
       </c>
       <c r="B6" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C6" t="s">
         <v>66</v>

</xml_diff>